<commit_message>
Add workbook structure comparison against baseline.
</commit_message>
<xml_diff>
--- a/data/incoming/FlowBI_Project_Management.xlsx
+++ b/data/incoming/FlowBI_Project_Management.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A16D45DF-E56B-4F7F-B65D-CBA0666B5CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1736383-D87A-48F2-A743-7CAC2BC343C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1738,118 +1738,118 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProjectsTable" displayName="ProjectsTable" ref="A1:L21" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProjectsTable" displayName="ProjectsTable" ref="A1:L21" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ProjectID" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ProjectName" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Department" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="ProjectManager" dataDxfId="72"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="City" dataDxfId="71"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Program" dataDxfId="70"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Priority" dataDxfId="69"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="StartDate" dataDxfId="68"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="PlannedEndDate" dataDxfId="67"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="BudgetSAR" dataDxfId="66"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="AsOfDate" dataDxfId="65"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="ProjectStatus" dataDxfId="64"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ProjectID" dataDxfId="73"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ProjectName" dataDxfId="72"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Department" dataDxfId="71"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="ProjectManager" dataDxfId="70"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="City" dataDxfId="69"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Program" dataDxfId="68"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Priority" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="StartDate" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="PlannedEndDate" dataDxfId="65"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="BudgetSAR" dataDxfId="64"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="AsOfDate" dataDxfId="63"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="ProjectStatus" dataDxfId="62"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="WeeklySnapshotsTable" displayName="WeeklySnapshotsTable" ref="A1:K541" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="WeeklySnapshotsTable" displayName="WeeklySnapshotsTable" ref="A1:K541" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="ProjectID" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="SnapshotDate" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="PlannedProgress" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="ActualProgress" dataDxfId="58"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="PlannedValueSAR" dataDxfId="57"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="EarnedValueSAR" dataDxfId="56"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="ActualCostSAR" dataDxfId="55"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="PeriodCostSAR" dataDxfId="54"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="EstimateToCompleteSAR" dataDxfId="53"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ScheduleDelayDays" dataDxfId="52"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="ScenarioNote" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="ProjectID" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="SnapshotDate" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="PlannedProgress" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="ActualProgress" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="PlannedValueSAR" dataDxfId="55"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="EarnedValueSAR" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="ActualCostSAR" dataDxfId="53"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="PeriodCostSAR" dataDxfId="52"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="EstimateToCompleteSAR" dataDxfId="51"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ScheduleDelayDays" dataDxfId="50"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="ScenarioNote" dataDxfId="49"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="TasksTable" displayName="TasksTable" ref="A1:M201" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="TasksTable" displayName="TasksTable" ref="A1:M201" totalsRowShown="0" headerRowDxfId="48" dataDxfId="47">
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="TaskID" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="ProjectID" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="TaskName" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Phase" dataDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Owner" dataDxfId="44"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="PlannedStart" dataDxfId="43"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="PlannedEnd" dataDxfId="42"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="ActualEnd" dataDxfId="41"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="TaskStatus" dataDxfId="40"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="CompletionPct" dataDxfId="39"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="PlannedHours" dataDxfId="38"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="ActualHours" dataDxfId="37"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0200-00000D000000}" name="Priority" dataDxfId="36"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="TaskID" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="ProjectID" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="TaskName" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Phase" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Owner" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="PlannedStart" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="PlannedEnd" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="ActualEnd" dataDxfId="39"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="TaskStatus" dataDxfId="38"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="CompletionPct" dataDxfId="37"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="PlannedHours" dataDxfId="36"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="ActualHours" dataDxfId="35"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0200-00000D000000}" name="Priority" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="RisksTable" displayName="RisksTable" ref="A1:L41" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="RisksTable" displayName="RisksTable" ref="A1:L41" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="RiskID" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="ProjectID" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="RiskDescription" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Category" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="ProbabilityScore" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="ImpactScore" dataDxfId="28"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="Owner" dataDxfId="27"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="OpenedDate" dataDxfId="26"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="ClosedDate" dataDxfId="25"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="RiskStatus" dataDxfId="24"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="Mitigation" dataDxfId="23"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="TargetActionDate" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="RiskID" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="ProjectID" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="RiskDescription" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Category" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="ProbabilityScore" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="ImpactScore" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="Owner" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="OpenedDate" dataDxfId="24"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="ClosedDate" dataDxfId="23"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="RiskStatus" dataDxfId="22"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="Mitigation" dataDxfId="21"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="TargetActionDate" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="CalendarTable" displayName="CalendarTable" ref="A1:E456" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="CalendarTable" displayName="CalendarTable" ref="A1:E456" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Date" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Year" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="MonthNumber" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="YearMonth" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Quarter" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Date" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Year" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="MonthNumber" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="YearMonth" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Quarter" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="ReadMeTable" displayName="ReadMeTable" ref="A1:B20" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="ReadMeTable" displayName="ReadMeTable" ref="A1:B20" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="البند / Item" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="التفاصيل / Details" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="البند / Item" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="التفاصيل / Details" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="ScenariosTable" displayName="ScenariosTable" ref="A1:G3" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="ScenariosTable" displayName="ScenariosTable" ref="A1:G3" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="ScenarioID" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="ProjectID" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="StartDate" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="EndDate" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Pattern" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="InjectedChange" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="ExpectedCheck" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="ScenarioID" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="ProjectID" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="StartDate" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="EndDate" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Pattern" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="InjectedChange" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="ExpectedCheck" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Detect Excel cell errors and flag formula review.
</commit_message>
<xml_diff>
--- a/data/incoming/FlowBI_Project_Management.xlsx
+++ b/data/incoming/FlowBI_Project_Management.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1736383-D87A-48F2-A743-7CAC2BC343C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D17E9608-D004-4566-AC1B-A045EA419917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,20 @@
     <sheet name="Scenarios" sheetId="7" r:id="rId7"/>
     <sheet name="Dictionary" sheetId="8" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>

<commit_message>
MONITOR: Dialog closure and newer check timestamp observed.
</commit_message>
<xml_diff>
--- a/data/incoming/FlowBI_Project_Management.xlsx
+++ b/data/incoming/FlowBI_Project_Management.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF8530E-70FD-462E-ADEF-5F40D6F3BE41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB40E421-BF95-43BE-A0A9-1F9A2AEDBE90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2149,7 +2149,7 @@
         <v>46207</v>
       </c>
       <c r="J2" s="8">
-        <v>500000</v>
+        <v>510000</v>
       </c>
       <c r="K2" s="7">
         <v>46312</v>

</xml_diff>

<commit_message>
Add reviewed correction preview and copy creation to desktop UI.
</commit_message>
<xml_diff>
--- a/data/incoming/FlowBI_Project_Management.xlsx
+++ b/data/incoming/FlowBI_Project_Management.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DDCAF88-77FA-44AA-BD81-5ED592A5EAD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D98FDA0-6EB6-4274-92D7-F8CE374CCD83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3169" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3169" uniqueCount="460">
   <si>
     <t>ProjectID</t>
   </si>
@@ -1417,6 +1417,9 @@
   </si>
   <si>
     <t>Calendar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completed </t>
   </si>
 </sst>
 </file>
@@ -2155,7 +2158,7 @@
         <v>46312</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>19</v>
+        <v>459</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1">

</xml_diff>

<commit_message>
Add correction audit records and ignore Excel lock files.
</commit_message>
<xml_diff>
--- a/data/incoming/FlowBI_Project_Management.xlsx
+++ b/data/incoming/FlowBI_Project_Management.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renad\flowguard-ai\data\incoming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D98FDA0-6EB6-4274-92D7-F8CE374CCD83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5DD964A-52CC-4AC8-9F4A-0A09B0960930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3169" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3169" uniqueCount="459">
   <si>
     <t>ProjectID</t>
   </si>
@@ -1417,9 +1417,6 @@
   </si>
   <si>
     <t>Calendar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Completed </t>
   </si>
 </sst>
 </file>
@@ -2158,7 +2155,7 @@
         <v>46312</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>459</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1">

</xml_diff>